<commit_message>
Update waypoint coordinates and add scripts for traffic scenario processing
</commit_message>
<xml_diff>
--- a/Deleted.xlsx
+++ b/Deleted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/jslagmolen_tudelft_nl/Documents/4321-15 ATM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{853A74F7-F05C-4285-894F-C741F98538CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF97F4AF-7F2F-4450-88B2-B0EA89C52315}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{853A74F7-F05C-4285-894F-C741F98538CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B4F0CFA-8CBE-4D20-94F2-E8CB47CBE966}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CF6879C-A2D4-4EBE-8E95-B361EE50E68E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="30">
   <si>
     <t>t</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>klm725</t>
   </si>
 </sst>
 </file>
@@ -495,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{583EB323-DF6E-42CF-8892-CA072A32C9AD}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -683,6 +686,11 @@
         <v>21</v>
       </c>
     </row>
+    <row r="21" spans="8:9" x14ac:dyDescent="0.3">
+      <c r="H21" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>